<commit_message>
Demo: result screenshots per product (click to enlarge); site-wide lightbox for product images; dashboard-style sample result workbooks (lab sync)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lab/samples/kalibre-lab-sample-result.xlsx
+++ b/lab/samples/kalibre-lab-sample-result.xlsx
@@ -1,41 +1,90 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <bookViews>
+    <workbookView activeTab="0"/>
+  </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
     <sheet name="Trades" sheetId="2" r:id="rId2"/>
+    <sheet name="Run" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trades'!$A$1:$J$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Run'!$A$1:$B$8</definedName>
+  </definedNames>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="0.00"/>
+    <numFmt numFmtId="166" formatCode="[Color10]+#,##0.00;[Red]-#,##0.00;0.00"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="6">
     <font>
-      <sz val="11"/>
+      <sz val="10"/>
+      <color rgb="FF1F2937"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="18"/>
+      <color rgb="FF1F2937"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF6B7280"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF6B7280"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF6B7280"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1F2937"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7F8FA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEF1F5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -43,277 +92,1446 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF4E79A7"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFE5E7EB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF4E79A7"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFE5E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFC7CDD6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF9CA3AF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="17">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" indent="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="1F2937"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="1F2937"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Balance after each trade (start 10,000)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Balance</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="22225" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="4E79A7"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Trades'!$A$2:$A$32</c:f>
+              <c:strCache>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>31</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Trades'!$J$2:$J$32</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>10200</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10270.379514871249</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10167.675719722536</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10371.029234116986</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>10267.318941775817</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10219.28946559044</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>10217.990565907534</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>10164.248594604265</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>10062.606108658223</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10263.858230831387</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10469.135395448015</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>10678.518103356975</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>10587.04367121349</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>10798.784544637761</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>10690.796699191384</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>10583.88873219947</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>10529.374245435409</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>10448.646233245996</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>10344.159770913537</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>10551.042966331806</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>10506.111086145893</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>10401.049975284435</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>10327.504891978851</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>10224.229843059064</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>10121.987544628473</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>10324.427295521042</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>10325.684734514965</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>10222.427887169815</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>10120.203608298118</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>10019.001572215137</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>9918.811556492985</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:marker val="1"/>
+        <c:axId val="5001"/>
+        <c:axId val="5002"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="5001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:spPr>
+          <a:ln w="6350">
+            <a:solidFill>
+              <a:srgbClr val="D1D5DB"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="6B7280"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="5002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:tickLblSkip val="5"/>
+        <c:tickMarkSkip val="5"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="5002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="9700"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="E5E7EB"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="6B7280"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="5001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="9525">
+      <a:solidFill>
+        <a:srgbClr val="E5E7EB"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr sz="900">
+          <a:latin typeface="Calibri"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="1F2937"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="1F2937"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Result of each trade (R)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>R</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4E79A7"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="4E79A7"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="4E79A7"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="4E79A7"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="6"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="7"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="8"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="9"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="4E79A7"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="10"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="4E79A7"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="11"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="4E79A7"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="12"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="13"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="4E79A7"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="14"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="15"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="16"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="17"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="18"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="19"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="4E79A7"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="20"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="21"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="22"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="23"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="24"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="25"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="4E79A7"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="26"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="4E79A7"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="27"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="28"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="29"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="30"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E15759"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Trades'!$A$2:$A$32</c:f>
+              <c:strCache>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>#1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>#2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>#3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>#4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>#5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>#6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>#7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>#8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>#9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>#10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>#11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>#12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>#13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>#14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>#15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>#16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>#17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>#18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>#19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>#20</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>#21</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>#22</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>#23</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>#24</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>#25</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>#26</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>#27</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>#28</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>#29</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>#30</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>#31</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Trades'!$I$2:$I$32</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="31"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.6899952438357783</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-0.9999999999999978</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.9999999999999993</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-1.0000000000000013</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-0.4677898530058625</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.012710273911710212</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-0.5259544032324639</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-0.9999999999999988</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.0000000000000013</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.999999999999992</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.0000000000000018</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-0.8566210335376763</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.0000000000000018</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-0.9999999999999948</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-0.9999999999999941</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-0.5150704825364468</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-0.7666933505038039</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-1</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1.9999999999999984</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>-0.42585249940967745</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>-0.9999999999999952</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>-0.7070928750495857</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>-1.0000000000000016</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>-0.9999999999999969</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>1.999999999999999</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.012179261453752714</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>-1.0000000000000004</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>-1</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>-0.9999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>-0.9999999999999989</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="55"/>
+        <c:axId val="5001"/>
+        <c:axId val="5002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="5001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:spPr>
+          <a:ln w="6350">
+            <a:solidFill>
+              <a:srgbClr val="D1D5DB"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="6B7280"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="5002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:tickLblSkip val="5"/>
+        <c:tickMarkSkip val="5"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="5002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="E5E7EB"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="6B7280"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="5001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="9525">
+      <a:solidFill>
+        <a:srgbClr val="E5E7EB"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr sz="900">
+          <a:latin typeface="Calibri"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B20"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FF4E79A7"/>
+  </sheetPr>
+  <dimension ref="A1:M26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="70" customWidth="1"/>
+    <col min="1" max="1" width="2" customWidth="1"/>
+    <col min="2" max="2" width="11.5" customWidth="1"/>
+    <col min="3" max="3" width="11.5" customWidth="1"/>
+    <col min="4" max="4" width="11.5" customWidth="1"/>
+    <col min="5" max="5" width="11.5" customWidth="1"/>
+    <col min="6" max="6" width="11.5" customWidth="1"/>
+    <col min="7" max="7" width="11.5" customWidth="1"/>
+    <col min="8" max="8" width="11.5" customWidth="1"/>
+    <col min="9" max="9" width="11.5" customWidth="1"/>
+    <col min="10" max="10" width="11.5" customWidth="1"/>
+    <col min="11" max="11" width="11.5" customWidth="1"/>
+    <col min="12" max="12" width="11.5" customWidth="1"/>
+    <col min="13" max="13" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Kalibre Lab: backtest of the sample rule on the sample prices</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Example.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Inputs</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kalibre-lab-sample-strategy.json + kalibre-lab-sample-prices.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Costs</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gross (no spread, commission or slippage)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">resultId</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">d75fe88a3f8370a53098995396c72b5cdb0a604643ac4ead53f3216bf1f94a79</t>
-        </is>
-      </c>
+    <row r="1" ht="28" customHeight="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kalibre Lab backtest</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Example · EMA trend rule on 3000 H1 bars · no costs · result ID kr1-d75fe88a3f8370a5</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trades</t>
+        </is>
+      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Win rate</t>
+        </is>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Profit factor</t>
+        </is>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Return</t>
+        </is>
+      </c>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max drawdown</t>
+        </is>
+      </c>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Expectancy (R)</t>
+        </is>
+      </c>
+      <c r="M4" s="3"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="B5" s="4">
+        <v>31</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="5">
+        <v>0.3225806451612903</v>
+      </c>
+      <c r="E5" s="5"/>
+      <c r="F5" s="6">
+        <v>0.9547231243792096</v>
+      </c>
+      <c r="G5" s="6"/>
+      <c r="H5" s="5">
+        <v>-0.008118844350701537</v>
+      </c>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5">
+        <v>0.08148815123658854</v>
+      </c>
+      <c r="K5" s="5"/>
+      <c r="L5" s="6">
+        <v>-0.01856807309347363</v>
+      </c>
+      <c r="M5" s="6"/>
     </row>
     <row r="6"/>
-    <row r="7">
-      <c r="A7" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Measure</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Trades</t>
-        </is>
-      </c>
-      <c r="B8" s="5">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Win rate</t>
-        </is>
-      </c>
-      <c r="B9" s="7">
-        <v>0.3225806451612903</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Expectancy (R)</t>
-        </is>
-      </c>
-      <c r="B10" s="8">
-        <v>-0.01856807309347363</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Average win (R)</t>
-        </is>
-      </c>
-      <c r="B11" s="8">
-        <v>1.6702174505289524</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Average loss (R)</t>
-        </is>
-      </c>
-      <c r="B12" s="8">
-        <v>-0.8227516557708194</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Profit factor</t>
-        </is>
-      </c>
-      <c r="B13" s="8">
-        <v>0.9547231243792096</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Return</t>
-        </is>
-      </c>
-      <c r="B14" s="7">
-        <v>-0.008118844350701537</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Max drawdown</t>
-        </is>
-      </c>
-      <c r="B15" s="7">
-        <v>0.08148815123658854</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Longest losing streak</t>
-        </is>
-      </c>
-      <c r="B16" s="5">
-        <v>5</v>
-      </c>
-    </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
     <row r="17"/>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The news filter is not applied in Quick Backtest (it needs the MT5 calendar).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Spread is assumed to be zero in Quick Backtest.</t>
-        </is>
-      </c>
-    </row>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25">
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The rule and the price series are examples. Download the rule file and the price file to run the same test in Kalibre Lab and get the same result ID.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
   </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="B25:M25"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I32"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FFC7CDD6"/>
+  </sheetPr>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="7" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="1" max="1" width="7" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="8" customWidth="1"/>
+    <col min="10" max="10" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr" s="1">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">#</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="1">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Side</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr" s="1">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Entry time</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Entry</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr" s="1">
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entry price</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Exit time</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Exit</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exit price</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Exit reason</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="1">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">P&amp;L</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">R</t>
         </is>
       </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Balance after</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2">
+      <c r="A2" s="10">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -326,7 +1544,7 @@
           <t xml:space="preserve">2030.01.14 17:00</t>
         </is>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="11">
         <v>99.73225</v>
       </c>
       <c r="E2" t="inlineStr">
@@ -334,7 +1552,7 @@
           <t xml:space="preserve">2030.01.14 20:00</t>
         </is>
       </c>
-      <c r="F2" s="6">
+      <c r="F2" s="11">
         <v>102.22107857142856</v>
       </c>
       <c r="G2" t="inlineStr">
@@ -342,15 +1560,18 @@
           <t xml:space="preserve">target</t>
         </is>
       </c>
-      <c r="H2" s="4">
+      <c r="H2" s="12">
         <v>200</v>
       </c>
-      <c r="I2" s="8">
+      <c r="I2" s="13">
         <v>2</v>
       </c>
+      <c r="J2" s="14">
+        <v>10200</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3">
+      <c r="A3" s="10">
         <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -363,7 +1584,7 @@
           <t xml:space="preserve">2030.01.17 19:00</t>
         </is>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="11">
         <v>101.40115</v>
       </c>
       <c r="E3" t="inlineStr">
@@ -371,7 +1592,7 @@
           <t xml:space="preserve">2030.01.21 04:00</t>
         </is>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="11">
         <v>100.23434142857144</v>
       </c>
       <c r="G3" t="inlineStr">
@@ -379,15 +1600,18 @@
           <t xml:space="preserve">trailing_stop</t>
         </is>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="12">
         <v>70.37951487124938</v>
       </c>
-      <c r="I3" s="8">
+      <c r="I3" s="13">
         <v>0.6899952438357783</v>
       </c>
+      <c r="J3" s="14">
+        <v>10270.379514871249</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4">
+      <c r="A4" s="10">
         <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -400,7 +1624,7 @@
           <t xml:space="preserve">2030.01.28 16:00</t>
         </is>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="11">
         <v>103.18994</v>
       </c>
       <c r="E4" t="inlineStr">
@@ -408,7 +1632,7 @@
           <t xml:space="preserve">2030.01.28 20:00</t>
         </is>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="11">
         <v>104.05275714285715</v>
       </c>
       <c r="G4" t="inlineStr">
@@ -416,15 +1640,18 @@
           <t xml:space="preserve">stop</t>
         </is>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="12">
         <v>-102.70379514871226</v>
       </c>
-      <c r="I4" s="8">
+      <c r="I4" s="13">
         <v>-0.9999999999999978</v>
       </c>
+      <c r="J4" s="14">
+        <v>10167.675719722536</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5">
+      <c r="A5" s="10">
         <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -437,7 +1664,7 @@
           <t xml:space="preserve">2030.02.04 10:00</t>
         </is>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="11">
         <v>93.8211</v>
       </c>
       <c r="E5" t="inlineStr">
@@ -445,7 +1672,7 @@
           <t xml:space="preserve">2030.02.05 09:00</t>
         </is>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="11">
         <v>83.71948571428572</v>
       </c>
       <c r="G5" t="inlineStr">
@@ -453,15 +1680,18 @@
           <t xml:space="preserve">target</t>
         </is>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="12">
         <v>203.35351439445066</v>
       </c>
-      <c r="I5" s="8">
+      <c r="I5" s="13">
         <v>1.9999999999999993</v>
       </c>
+      <c r="J5" s="14">
+        <v>10371.029234116986</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6">
+      <c r="A6" s="10">
         <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -474,7 +1704,7 @@
           <t xml:space="preserve">2030.02.11 14:00</t>
         </is>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="11">
         <v>91.754</v>
       </c>
       <c r="E6" t="inlineStr">
@@ -482,7 +1712,7 @@
           <t xml:space="preserve">2030.02.11 15:00</t>
         </is>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="11">
         <v>94.55340714285715</v>
       </c>
       <c r="G6" t="inlineStr">
@@ -490,15 +1720,18 @@
           <t xml:space="preserve">stop</t>
         </is>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="12">
         <v>-103.71029234117002</v>
       </c>
-      <c r="I6" s="8">
+      <c r="I6" s="13">
         <v>-1.0000000000000013</v>
       </c>
+      <c r="J6" s="14">
+        <v>10267.318941775817</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7">
+      <c r="A7" s="10">
         <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
@@ -511,7 +1744,7 @@
           <t xml:space="preserve">2030.02.11 17:00</t>
         </is>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="11">
         <v>100.33304</v>
       </c>
       <c r="E7" t="inlineStr">
@@ -519,7 +1752,7 @@
           <t xml:space="preserve">2030.02.12 05:00</t>
         </is>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="11">
         <v>98.42329928571428</v>
       </c>
       <c r="G7" t="inlineStr">
@@ -527,15 +1760,18 @@
           <t xml:space="preserve">trailing_stop</t>
         </is>
       </c>
-      <c r="H7" s="4">
+      <c r="H7" s="12">
         <v>-48.02947618537617</v>
       </c>
-      <c r="I7" s="8">
+      <c r="I7" s="13">
         <v>-0.4677898530058625</v>
       </c>
+      <c r="J7" s="14">
+        <v>10219.28946559044</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8">
+      <c r="A8" s="10">
         <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
@@ -548,7 +1784,7 @@
           <t xml:space="preserve">2030.02.12 19:00</t>
         </is>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="11">
         <v>96.15702</v>
       </c>
       <c r="E8" t="inlineStr">
@@ -556,7 +1792,7 @@
           <t xml:space="preserve">2030.02.13 14:00</t>
         </is>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="11">
         <v>96.19746071428571</v>
       </c>
       <c r="G8" t="inlineStr">
@@ -564,15 +1800,18 @@
           <t xml:space="preserve">trailing_stop</t>
         </is>
       </c>
-      <c r="H8" s="4">
+      <c r="H8" s="12">
         <v>-1.2988996829070913</v>
       </c>
-      <c r="I8" s="8">
+      <c r="I8" s="13">
         <v>-0.012710273911710212</v>
       </c>
+      <c r="J8" s="14">
+        <v>10217.990565907534</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9">
+      <c r="A9" s="10">
         <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
@@ -585,7 +1824,7 @@
           <t xml:space="preserve">2030.02.13 19:00</t>
         </is>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="11">
         <v>106.31861</v>
       </c>
       <c r="E9" t="inlineStr">
@@ -593,7 +1832,7 @@
           <t xml:space="preserve">2030.02.13 23:00</t>
         </is>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="11">
         <v>104.38021857142856</v>
       </c>
       <c r="G9" t="inlineStr">
@@ -601,15 +1840,18 @@
           <t xml:space="preserve">trailing_stop</t>
         </is>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="12">
         <v>-53.741971303268436</v>
       </c>
-      <c r="I9" s="8">
+      <c r="I9" s="13">
         <v>-0.5259544032324639</v>
       </c>
+      <c r="J9" s="14">
+        <v>10164.248594604265</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10">
+      <c r="A10" s="10">
         <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
@@ -622,7 +1864,7 @@
           <t xml:space="preserve">2030.02.28 09:00</t>
         </is>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="11">
         <v>121.91674</v>
       </c>
       <c r="E10" t="inlineStr">
@@ -630,7 +1872,7 @@
           <t xml:space="preserve">2030.02.28 11:00</t>
         </is>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="11">
         <v>123.53398714285714</v>
       </c>
       <c r="G10" t="inlineStr">
@@ -638,15 +1880,18 @@
           <t xml:space="preserve">stop</t>
         </is>
       </c>
-      <c r="H10" s="4">
+      <c r="H10" s="12">
         <v>-101.64248594604253</v>
       </c>
-      <c r="I10" s="8">
+      <c r="I10" s="13">
         <v>-0.9999999999999988</v>
       </c>
+      <c r="J10" s="14">
+        <v>10062.606108658223</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11">
+      <c r="A11" s="10">
         <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
@@ -659,7 +1904,7 @@
           <t xml:space="preserve">2030.02.28 12:00</t>
         </is>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="11">
         <v>123.24134</v>
       </c>
       <c r="E11" t="inlineStr">
@@ -667,7 +1912,7 @@
           <t xml:space="preserve">2030.02.28 15:00</t>
         </is>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="11">
         <v>126.54801142857141</v>
       </c>
       <c r="G11" t="inlineStr">
@@ -675,15 +1920,18 @@
           <t xml:space="preserve">target</t>
         </is>
       </c>
-      <c r="H11" s="4">
+      <c r="H11" s="12">
         <v>201.25212217316457</v>
       </c>
-      <c r="I11" s="8">
+      <c r="I11" s="13">
         <v>2.0000000000000013</v>
       </c>
+      <c r="J11" s="14">
+        <v>10263.858230831387</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12">
+      <c r="A12" s="10">
         <v>11</v>
       </c>
       <c r="B12" t="inlineStr">
@@ -696,7 +1944,7 @@
           <t xml:space="preserve">2030.03.06 13:00</t>
         </is>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="11">
         <v>126.49166</v>
       </c>
       <c r="E12" t="inlineStr">
@@ -704,7 +1952,7 @@
           <t xml:space="preserve">2030.03.06 20:00</t>
         </is>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="11">
         <v>129.40453428571428</v>
       </c>
       <c r="G12" t="inlineStr">
@@ -712,15 +1960,18 @@
           <t xml:space="preserve">target</t>
         </is>
       </c>
-      <c r="H12" s="4">
+      <c r="H12" s="12">
         <v>205.27716461662692</v>
       </c>
-      <c r="I12" s="8">
+      <c r="I12" s="13">
         <v>1.999999999999992</v>
       </c>
+      <c r="J12" s="14">
+        <v>10469.135395448015</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13">
+      <c r="A13" s="10">
         <v>12</v>
       </c>
       <c r="B13" t="inlineStr">
@@ -733,7 +1984,7 @@
           <t xml:space="preserve">2030.03.21 13:00</t>
         </is>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="11">
         <v>118.418</v>
       </c>
       <c r="E13" t="inlineStr">
@@ -741,7 +1992,7 @@
           <t xml:space="preserve">2030.03.21 21:00</t>
         </is>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="11">
         <v>110.97886285714286</v>
       </c>
       <c r="G13" t="inlineStr">
@@ -749,15 +2000,18 @@
           <t xml:space="preserve">target</t>
         </is>
       </c>
-      <c r="H13" s="4">
+      <c r="H13" s="12">
         <v>209.38270790896047</v>
       </c>
-      <c r="I13" s="8">
+      <c r="I13" s="13">
         <v>2.0000000000000018</v>
       </c>
+      <c r="J13" s="14">
+        <v>10678.518103356975</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14">
+      <c r="A14" s="10">
         <v>13</v>
       </c>
       <c r="B14" t="inlineStr">
@@ -770,7 +2024,7 @@
           <t xml:space="preserve">2030.04.03 18:00</t>
         </is>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="11">
         <v>94.72088</v>
       </c>
       <c r="E14" t="inlineStr">
@@ -778,7 +2032,7 @@
           <t xml:space="preserve">2030.04.04 01:00</t>
         </is>
       </c>
-      <c r="F14" s="6">
+      <c r="F14" s="11">
         <v>93.64078</v>
       </c>
       <c r="G14" t="inlineStr">
@@ -786,15 +2040,18 @@
           <t xml:space="preserve">opposite_signal</t>
         </is>
       </c>
-      <c r="H14" s="4">
+      <c r="H14" s="12">
         <v>-91.47443214348439</v>
       </c>
-      <c r="I14" s="8">
+      <c r="I14" s="13">
         <v>-0.8566210335376763</v>
       </c>
+      <c r="J14" s="14">
+        <v>10587.04367121349</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15">
+      <c r="A15" s="10">
         <v>14</v>
       </c>
       <c r="B15" t="inlineStr">
@@ -807,7 +2064,7 @@
           <t xml:space="preserve">2030.04.11 14:00</t>
         </is>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="11">
         <v>95.93045</v>
       </c>
       <c r="E15" t="inlineStr">
@@ -815,7 +2072,7 @@
           <t xml:space="preserve">2030.04.12 22:00</t>
         </is>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="11">
         <v>93.53361285714286</v>
       </c>
       <c r="G15" t="inlineStr">
@@ -823,15 +2080,18 @@
           <t xml:space="preserve">target</t>
         </is>
       </c>
-      <c r="H15" s="4">
+      <c r="H15" s="12">
         <v>211.74087342426998</v>
       </c>
-      <c r="I15" s="8">
+      <c r="I15" s="13">
         <v>2.0000000000000018</v>
       </c>
+      <c r="J15" s="14">
+        <v>10798.784544637761</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16">
+      <c r="A16" s="10">
         <v>15</v>
       </c>
       <c r="B16" t="inlineStr">
@@ -844,7 +2104,7 @@
           <t xml:space="preserve">2030.04.15 12:00</t>
         </is>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="11">
         <v>97.08096</v>
       </c>
       <c r="E16" t="inlineStr">
@@ -852,7 +2112,7 @@
           <t xml:space="preserve">2030.04.15 15:00</t>
         </is>
       </c>
-      <c r="F16" s="6">
+      <c r="F16" s="11">
         <v>95.93626</v>
       </c>
       <c r="G16" t="inlineStr">
@@ -860,15 +2120,18 @@
           <t xml:space="preserve">stop</t>
         </is>
       </c>
-      <c r="H16" s="4">
+      <c r="H16" s="12">
         <v>-107.98784544637705</v>
       </c>
-      <c r="I16" s="8">
+      <c r="I16" s="13">
         <v>-0.9999999999999948</v>
       </c>
+      <c r="J16" s="14">
+        <v>10690.796699191384</v>
+      </c>
     </row>
     <row r="17">
-      <c r="A17">
+      <c r="A17" s="10">
         <v>16</v>
       </c>
       <c r="B17" t="inlineStr">
@@ -881,7 +2144,7 @@
           <t xml:space="preserve">2030.04.16 12:00</t>
         </is>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="11">
         <v>96.64454</v>
       </c>
       <c r="E17" t="inlineStr">
@@ -889,7 +2152,7 @@
           <t xml:space="preserve">2030.04.16 16:00</t>
         </is>
       </c>
-      <c r="F17" s="6">
+      <c r="F17" s="11">
         <v>95.62849000000001</v>
       </c>
       <c r="G17" t="inlineStr">
@@ -897,15 +2160,18 @@
           <t xml:space="preserve">stop</t>
         </is>
       </c>
-      <c r="H17" s="4">
+      <c r="H17" s="12">
         <v>-106.90796699191321</v>
       </c>
-      <c r="I17" s="8">
+      <c r="I17" s="13">
         <v>-0.9999999999999941</v>
       </c>
+      <c r="J17" s="14">
+        <v>10583.88873219947</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18">
+      <c r="A18" s="10">
         <v>17</v>
       </c>
       <c r="B18" t="inlineStr">
@@ -918,7 +2184,7 @@
           <t xml:space="preserve">2030.04.17 10:00</t>
         </is>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="11">
         <v>95.84433</v>
       </c>
       <c r="E18" t="inlineStr">
@@ -926,7 +2192,7 @@
           <t xml:space="preserve">2030.04.17 14:00</t>
         </is>
       </c>
-      <c r="F18" s="6">
+      <c r="F18" s="11">
         <v>95.18971</v>
       </c>
       <c r="G18" t="inlineStr">
@@ -934,15 +2200,18 @@
           <t xml:space="preserve">opposite_signal</t>
         </is>
       </c>
-      <c r="H18" s="4">
+      <c r="H18" s="12">
         <v>-54.514486764060436</v>
       </c>
-      <c r="I18" s="8">
+      <c r="I18" s="13">
         <v>-0.5150704825364468</v>
       </c>
+      <c r="J18" s="14">
+        <v>10529.374245435409</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19">
+      <c r="A19" s="10">
         <v>18</v>
       </c>
       <c r="B19" t="inlineStr">
@@ -955,7 +2224,7 @@
           <t xml:space="preserve">2030.04.17 14:00</t>
         </is>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="11">
         <v>95.18971</v>
       </c>
       <c r="E19" t="inlineStr">
@@ -963,7 +2232,7 @@
           <t xml:space="preserve">2030.04.17 22:00</t>
         </is>
       </c>
-      <c r="F19" s="6">
+      <c r="F19" s="11">
         <v>96.07084</v>
       </c>
       <c r="G19" t="inlineStr">
@@ -971,15 +2240,18 @@
           <t xml:space="preserve">opposite_signal</t>
         </is>
       </c>
-      <c r="H19" s="4">
+      <c r="H19" s="12">
         <v>-80.72801218941338</v>
       </c>
-      <c r="I19" s="8">
+      <c r="I19" s="13">
         <v>-0.7666933505038039</v>
       </c>
+      <c r="J19" s="14">
+        <v>10448.646233245996</v>
+      </c>
     </row>
     <row r="20">
-      <c r="A20">
+      <c r="A20" s="10">
         <v>19</v>
       </c>
       <c r="B20" t="inlineStr">
@@ -992,7 +2264,7 @@
           <t xml:space="preserve">2030.04.30 13:00</t>
         </is>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="11">
         <v>100.14651</v>
       </c>
       <c r="E20" t="inlineStr">
@@ -1000,7 +2272,7 @@
           <t xml:space="preserve">2030.04.30 14:00</t>
         </is>
       </c>
-      <c r="F20" s="6">
+      <c r="F20" s="11">
         <v>98.77568714285715</v>
       </c>
       <c r="G20" t="inlineStr">
@@ -1008,15 +2280,18 @@
           <t xml:space="preserve">stop</t>
         </is>
       </c>
-      <c r="H20" s="4">
+      <c r="H20" s="12">
         <v>-104.48646233245996</v>
       </c>
-      <c r="I20" s="8">
+      <c r="I20" s="13">
         <v>-1</v>
       </c>
+      <c r="J20" s="14">
+        <v>10344.159770913537</v>
+      </c>
     </row>
     <row r="21">
-      <c r="A21">
+      <c r="A21" s="10">
         <v>20</v>
       </c>
       <c r="B21" t="inlineStr">
@@ -1029,7 +2304,7 @@
           <t xml:space="preserve">2030.05.07 13:00</t>
         </is>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="11">
         <v>105.73824</v>
       </c>
       <c r="E21" t="inlineStr">
@@ -1037,7 +2312,7 @@
           <t xml:space="preserve">2030.05.08 03:00</t>
         </is>
       </c>
-      <c r="F21" s="6">
+      <c r="F21" s="11">
         <v>108.64477142857143</v>
       </c>
       <c r="G21" t="inlineStr">
@@ -1045,15 +2320,18 @@
           <t xml:space="preserve">target</t>
         </is>
       </c>
-      <c r="H21" s="4">
+      <c r="H21" s="12">
         <v>206.88319541827056</v>
       </c>
-      <c r="I21" s="8">
+      <c r="I21" s="13">
         <v>1.9999999999999984</v>
       </c>
+      <c r="J21" s="14">
+        <v>10551.042966331806</v>
+      </c>
     </row>
     <row r="22">
-      <c r="A22">
+      <c r="A22" s="10">
         <v>21</v>
       </c>
       <c r="B22" t="inlineStr">
@@ -1066,7 +2344,7 @@
           <t xml:space="preserve">2030.05.09 12:00</t>
         </is>
       </c>
-      <c r="D22" s="6">
+      <c r="D22" s="11">
         <v>103.9365</v>
       </c>
       <c r="E22" t="inlineStr">
@@ -1074,7 +2352,7 @@
           <t xml:space="preserve">2030.05.09 21:00</t>
         </is>
       </c>
-      <c r="F22" s="6">
+      <c r="F22" s="11">
         <v>104.62955</v>
       </c>
       <c r="G22" t="inlineStr">
@@ -1082,15 +2360,18 @@
           <t xml:space="preserve">trailing_stop</t>
         </is>
       </c>
-      <c r="H22" s="4">
+      <c r="H22" s="12">
         <v>-44.93188018591297</v>
       </c>
-      <c r="I22" s="8">
+      <c r="I22" s="13">
         <v>-0.42585249940967745</v>
       </c>
+      <c r="J22" s="14">
+        <v>10506.111086145893</v>
+      </c>
     </row>
     <row r="23">
-      <c r="A23">
+      <c r="A23" s="10">
         <v>22</v>
       </c>
       <c r="B23" t="inlineStr">
@@ -1103,7 +2384,7 @@
           <t xml:space="preserve">2030.05.31 09:00</t>
         </is>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="11">
         <v>113.14837</v>
       </c>
       <c r="E23" t="inlineStr">
@@ -1111,7 +2392,7 @@
           <t xml:space="preserve">2030.05.31 10:00</t>
         </is>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="11">
         <v>111.88734428571429</v>
       </c>
       <c r="G23" t="inlineStr">
@@ -1119,15 +2400,18 @@
           <t xml:space="preserve">stop</t>
         </is>
       </c>
-      <c r="H23" s="4">
+      <c r="H23" s="12">
         <v>-105.06111086145842</v>
       </c>
-      <c r="I23" s="8">
+      <c r="I23" s="13">
         <v>-0.9999999999999952</v>
       </c>
+      <c r="J23" s="14">
+        <v>10401.049975284435</v>
+      </c>
     </row>
     <row r="24">
-      <c r="A24">
+      <c r="A24" s="10">
         <v>23</v>
       </c>
       <c r="B24" t="inlineStr">
@@ -1140,7 +2424,7 @@
           <t xml:space="preserve">2030.05.31 12:00</t>
         </is>
       </c>
-      <c r="D24" s="6">
+      <c r="D24" s="11">
         <v>110.5711</v>
       </c>
       <c r="E24" t="inlineStr">
@@ -1148,7 +2432,7 @@
           <t xml:space="preserve">2030.05.31 14:00</t>
         </is>
       </c>
-      <c r="F24" s="6">
+      <c r="F24" s="11">
         <v>111.52847142857142</v>
       </c>
       <c r="G24" t="inlineStr">
@@ -1156,15 +2440,18 @@
           <t xml:space="preserve">trailing_stop</t>
         </is>
       </c>
-      <c r="H24" s="4">
+      <c r="H24" s="12">
         <v>-73.54508330558293</v>
       </c>
-      <c r="I24" s="8">
+      <c r="I24" s="13">
         <v>-0.7070928750495857</v>
       </c>
+      <c r="J24" s="14">
+        <v>10327.504891978851</v>
+      </c>
     </row>
     <row r="25">
-      <c r="A25">
+      <c r="A25" s="10">
         <v>24</v>
       </c>
       <c r="B25" t="inlineStr">
@@ -1177,7 +2464,7 @@
           <t xml:space="preserve">2030.06.04 16:00</t>
         </is>
       </c>
-      <c r="D25" s="6">
+      <c r="D25" s="11">
         <v>113.10392</v>
       </c>
       <c r="E25" t="inlineStr">
@@ -1185,7 +2472,7 @@
           <t xml:space="preserve">2030.06.04 20:00</t>
         </is>
       </c>
-      <c r="F25" s="6">
+      <c r="F25" s="11">
         <v>111.92225</v>
       </c>
       <c r="G25" t="inlineStr">
@@ -1193,15 +2480,18 @@
           <t xml:space="preserve">stop</t>
         </is>
       </c>
-      <c r="H25" s="4">
+      <c r="H25" s="12">
         <v>-103.27504891978869</v>
       </c>
-      <c r="I25" s="8">
+      <c r="I25" s="13">
         <v>-1.0000000000000016</v>
       </c>
+      <c r="J25" s="14">
+        <v>10224.229843059064</v>
+      </c>
     </row>
     <row r="26">
-      <c r="A26">
+      <c r="A26" s="10">
         <v>25</v>
       </c>
       <c r="B26" t="inlineStr">
@@ -1214,7 +2504,7 @@
           <t xml:space="preserve">2030.06.10 13:00</t>
         </is>
       </c>
-      <c r="D26" s="6">
+      <c r="D26" s="11">
         <v>117.01259</v>
       </c>
       <c r="E26" t="inlineStr">
@@ -1222,7 +2512,7 @@
           <t xml:space="preserve">2030.06.10 23:00</t>
         </is>
       </c>
-      <c r="F26" s="6">
+      <c r="F26" s="11">
         <v>115.71205714285715</v>
       </c>
       <c r="G26" t="inlineStr">
@@ -1230,15 +2520,18 @@
           <t xml:space="preserve">stop</t>
         </is>
       </c>
-      <c r="H26" s="4">
+      <c r="H26" s="12">
         <v>-102.24229843059032</v>
       </c>
-      <c r="I26" s="8">
+      <c r="I26" s="13">
         <v>-0.9999999999999969</v>
       </c>
+      <c r="J26" s="14">
+        <v>10121.987544628473</v>
+      </c>
     </row>
     <row r="27">
-      <c r="A27">
+      <c r="A27" s="10">
         <v>26</v>
       </c>
       <c r="B27" t="inlineStr">
@@ -1251,7 +2544,7 @@
           <t xml:space="preserve">2030.06.11 14:00</t>
         </is>
       </c>
-      <c r="D27" s="6">
+      <c r="D27" s="11">
         <v>116.65727</v>
       </c>
       <c r="E27" t="inlineStr">
@@ -1259,7 +2552,7 @@
           <t xml:space="preserve">2030.06.12 20:00</t>
         </is>
       </c>
-      <c r="F27" s="6">
+      <c r="F27" s="11">
         <v>127.06659571428571</v>
       </c>
       <c r="G27" t="inlineStr">
@@ -1267,15 +2560,18 @@
           <t xml:space="preserve">target</t>
         </is>
       </c>
-      <c r="H27" s="4">
+      <c r="H27" s="12">
         <v>202.43975089256935</v>
       </c>
-      <c r="I27" s="8">
+      <c r="I27" s="13">
         <v>1.999999999999999</v>
       </c>
+      <c r="J27" s="14">
+        <v>10324.427295521042</v>
+      </c>
     </row>
     <row r="28">
-      <c r="A28">
+      <c r="A28" s="10">
         <v>27</v>
       </c>
       <c r="B28" t="inlineStr">
@@ -1288,7 +2584,7 @@
           <t xml:space="preserve">2030.06.13 14:00</t>
         </is>
       </c>
-      <c r="D28" s="6">
+      <c r="D28" s="11">
         <v>114.22148</v>
       </c>
       <c r="E28" t="inlineStr">
@@ -1296,7 +2592,7 @@
           <t xml:space="preserve">2030.06.14 09:00</t>
         </is>
       </c>
-      <c r="F28" s="6">
+      <c r="F28" s="11">
         <v>114.16169357142857</v>
       </c>
       <c r="G28" t="inlineStr">
@@ -1304,15 +2600,18 @@
           <t xml:space="preserve">trailing_stop</t>
         </is>
       </c>
-      <c r="H28" s="4">
+      <c r="H28" s="12">
         <v>1.2574389939241182</v>
       </c>
-      <c r="I28" s="8">
+      <c r="I28" s="13">
         <v>0.012179261453752714</v>
       </c>
+      <c r="J28" s="14">
+        <v>10325.684734514965</v>
+      </c>
     </row>
     <row r="29">
-      <c r="A29">
+      <c r="A29" s="10">
         <v>28</v>
       </c>
       <c r="B29" t="inlineStr">
@@ -1325,7 +2624,7 @@
           <t xml:space="preserve">2030.06.19 12:00</t>
         </is>
       </c>
-      <c r="D29" s="6">
+      <c r="D29" s="11">
         <v>120.93796</v>
       </c>
       <c r="E29" t="inlineStr">
@@ -1333,7 +2632,7 @@
           <t xml:space="preserve">2030.06.19 18:00</t>
         </is>
       </c>
-      <c r="F29" s="6">
+      <c r="F29" s="11">
         <v>126.60270000000001</v>
       </c>
       <c r="G29" t="inlineStr">
@@ -1341,15 +2640,18 @@
           <t xml:space="preserve">stop</t>
         </is>
       </c>
-      <c r="H29" s="4">
+      <c r="H29" s="12">
         <v>-103.2568473451497</v>
       </c>
-      <c r="I29" s="8">
+      <c r="I29" s="13">
         <v>-1.0000000000000004</v>
       </c>
+      <c r="J29" s="14">
+        <v>10222.427887169815</v>
+      </c>
     </row>
     <row r="30">
-      <c r="A30">
+      <c r="A30" s="10">
         <v>29</v>
       </c>
       <c r="B30" t="inlineStr">
@@ -1362,7 +2664,7 @@
           <t xml:space="preserve">2030.06.21 09:00</t>
         </is>
       </c>
-      <c r="D30" s="6">
+      <c r="D30" s="11">
         <v>123.99532</v>
       </c>
       <c r="E30" t="inlineStr">
@@ -1370,7 +2672,7 @@
           <t xml:space="preserve">2030.06.21 12:00</t>
         </is>
       </c>
-      <c r="F30" s="6">
+      <c r="F30" s="11">
         <v>119.99406571428572</v>
       </c>
       <c r="G30" t="inlineStr">
@@ -1378,15 +2680,18 @@
           <t xml:space="preserve">stop</t>
         </is>
       </c>
-      <c r="H30" s="4">
+      <c r="H30" s="12">
         <v>-102.22427887169815</v>
       </c>
-      <c r="I30" s="8">
+      <c r="I30" s="13">
         <v>-1</v>
       </c>
+      <c r="J30" s="14">
+        <v>10120.203608298118</v>
+      </c>
     </row>
     <row r="31">
-      <c r="A31">
+      <c r="A31" s="10">
         <v>30</v>
       </c>
       <c r="B31" t="inlineStr">
@@ -1399,7 +2704,7 @@
           <t xml:space="preserve">2030.06.25 19:00</t>
         </is>
       </c>
-      <c r="D31" s="6">
+      <c r="D31" s="11">
         <v>116.60581</v>
       </c>
       <c r="E31" t="inlineStr">
@@ -1407,7 +2712,7 @@
           <t xml:space="preserve">2030.06.25 22:00</t>
         </is>
       </c>
-      <c r="F31" s="6">
+      <c r="F31" s="11">
         <v>120.73044142857144</v>
       </c>
       <c r="G31" t="inlineStr">
@@ -1415,15 +2720,18 @@
           <t xml:space="preserve">stop</t>
         </is>
       </c>
-      <c r="H31" s="4">
+      <c r="H31" s="12">
         <v>-101.20203608298114</v>
       </c>
-      <c r="I31" s="8">
+      <c r="I31" s="13">
         <v>-0.9999999999999996</v>
       </c>
+      <c r="J31" s="14">
+        <v>10019.001572215137</v>
+      </c>
     </row>
     <row r="32">
-      <c r="A32">
+      <c r="A32" s="10">
         <v>31</v>
       </c>
       <c r="B32" t="inlineStr">
@@ -1436,7 +2744,7 @@
           <t xml:space="preserve">2030.06.27 17:00</t>
         </is>
       </c>
-      <c r="D32" s="6">
+      <c r="D32" s="11">
         <v>127.93646</v>
       </c>
       <c r="E32" t="inlineStr">
@@ -1444,7 +2752,7 @@
           <t xml:space="preserve">2030.06.27 17:00</t>
         </is>
       </c>
-      <c r="F32" s="6">
+      <c r="F32" s="11">
         <v>122.71377</v>
       </c>
       <c r="G32" t="inlineStr">
@@ -1452,13 +2760,150 @@
           <t xml:space="preserve">stop</t>
         </is>
       </c>
-      <c r="H32" s="4">
+      <c r="H32" s="12">
         <v>-100.19001572215126</v>
       </c>
-      <c r="I32" s="8">
+      <c r="I32" s="13">
         <v>-0.9999999999999989</v>
       </c>
+      <c r="J32" s="14">
+        <v>9918.811556492985</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total</t>
+        </is>
+      </c>
+      <c r="B33" s="15"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
+      <c r="H33" s="16">
+        <v>-81.18844350701237</v>
+      </c>
+      <c r="I33" s="15"/>
+      <c r="J33" s="16"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J32"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FFC7CDD6"/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="80" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Item</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rule file</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kalibre-lab-sample-strategy.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Price file</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kalibre-lab-sample-prices.csv (3000 H1 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Costs</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None (spread, commission and slippage set to 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Result ID</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d75fe88a3f8370a53098995396c72b5cdb0a604643ac4ead53f3216bf1f94a79</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Engine version</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.2.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Note</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The news filter is not applied in a quick backtest (it needs the MT5 calendar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Note</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The spread is assumed to be zero in a quick backtest.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B8"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>